<commit_message>
working on naukri 5 registarion scenario, data driven testing assignment 15 day 19 concepts- in progress not completed
</commit_message>
<xml_diff>
--- a/M18_qclass/Assignments/datasets_excels/data.xlsx
+++ b/M18_qclass/Assignments/datasets_excels/data.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D21C90-A319-4A41-8136-7E8369FB87FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3430497F-894F-4A27-8493-6691E4C108D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
   <si>
     <t>admin_username</t>
   </si>
@@ -98,13 +98,76 @@
   </si>
   <si>
     <t>selenium@122</t>
+  </si>
+  <si>
+    <t>fullName</t>
+  </si>
+  <si>
+    <t>emaiID</t>
+  </si>
+  <si>
+    <t>mobileNo</t>
+  </si>
+  <si>
+    <t>workStatus</t>
+  </si>
+  <si>
+    <t>VarunA</t>
+  </si>
+  <si>
+    <t>VarunB</t>
+  </si>
+  <si>
+    <t>VarunC</t>
+  </si>
+  <si>
+    <t>VarunD</t>
+  </si>
+  <si>
+    <t>VarunE</t>
+  </si>
+  <si>
+    <t>varuna@gmail.com</t>
+  </si>
+  <si>
+    <t>varunb@gmail.com</t>
+  </si>
+  <si>
+    <t>varunc@gmail.com</t>
+  </si>
+  <si>
+    <t>varund@gmail.com</t>
+  </si>
+  <si>
+    <t>varune@gmail.com</t>
+  </si>
+  <si>
+    <t>VarunA@123</t>
+  </si>
+  <si>
+    <t>VarunC@123</t>
+  </si>
+  <si>
+    <t>VarunD@123</t>
+  </si>
+  <si>
+    <t>VarunE@123</t>
+  </si>
+  <si>
+    <t>VarunB@123</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,6 +195,18 @@
       <color theme="10"/>
       <name val="Jetbra"/>
     </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF6F737A"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -154,7 +229,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -165,6 +240,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -595,9 +674,136 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="22.5546875" customWidth="1"/>
+    <col min="3" max="3" width="25.21875" customWidth="1"/>
+    <col min="4" max="4" width="19.5546875" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2">
+        <v>9123123121</v>
+      </c>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D3">
+        <v>8123123122</v>
+      </c>
+      <c r="E3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D4">
+        <v>7123123123</v>
+      </c>
+      <c r="E4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5">
+        <v>6123123124</v>
+      </c>
+      <c r="E5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6">
+        <v>9123123125</v>
+      </c>
+      <c r="E6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{B12FB8A9-09A8-4872-A0EE-A5FFAE7D62BF}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{7AD10E12-D6DC-45A4-A21D-A13B684ADCCC}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{DCD279A5-FEA9-4D57-A37A-DE761B312BDE}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{E14157B6-0A8C-4AD9-A424-D88AA2E4B6AA}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{E0584B77-3019-44C7-B0E5-1FF43BEBC5C5}"/>
+    <hyperlink ref="C2" r:id="rId6" xr:uid="{2FB99858-7EB5-4C7A-AF35-02CC14DD5E44}"/>
+    <hyperlink ref="C3" r:id="rId7" xr:uid="{77824B32-128F-422C-808C-9CA01CA69890}"/>
+    <hyperlink ref="C4" r:id="rId8" xr:uid="{59DE1ADB-9511-4DA0-AACB-1652A7EE21AA}"/>
+    <hyperlink ref="C6" r:id="rId9" xr:uid="{C34AA77F-4FEC-4135-9566-4B4146EA5756}"/>
+    <hyperlink ref="C5" r:id="rId10" xr:uid="{B5CE53B4-DA1B-4B31-A6B0-55288F401C1C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>